<commit_message>
all 6799 frames run
</commit_message>
<xml_diff>
--- a/results/ch2_permation_residue_comb.xlsx
+++ b/results/ch2_permation_residue_comb.xlsx
@@ -453,40 +453,40 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>98, 423, 780, 1105</t>
+          <t>98, 130, 748, 1073</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>780</t>
+          <t>130, 130</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5552</t>
+          <t>5178, 5582</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>98, 130, 748, 1073</t>
+          <t>98, 423, 780, 1105</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>130, 130</t>
+          <t>780</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5178, 5582</t>
+          <t>5552</t>
         </is>
       </c>
     </row>

</xml_diff>